<commit_message>
Numpy 2.4 casting error fix Improved documentation with more references and examples including the results files Transfer function scan allows for multi-frequency perturbations Time and frequency domain graphs during startup and selected perturbations Clean up of functions and generalization for admittance calculation and Bode plots
</commit_message>
<xml_diff>
--- a/Examples/Energy_hub/toplogy_hub.xlsx
+++ b/Examples/Energy_hub/toplogy_hub.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fcifuent\PycharmProjects\Z-tool\Examples\Energy Hub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fcifuent\GitLab Projects\Z-tool\Examples\Energy_hub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08867DED-DAA0-4CFD-B59A-1EA211F4C10D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19EA660-C86D-43D1-BD74-D9EA610205A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5205" yWindow="3255" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test_case" sheetId="1" r:id="rId1"/>
+    <sheet name="test_case3" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
   <si>
     <t>g1-1</t>
   </si>
@@ -481,12 +482,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S19"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -542,7 +543,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -601,7 +602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -660,7 +661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -719,7 +720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -739,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="2">
         <v>0</v>
@@ -754,7 +755,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5" s="2">
         <v>0</v>
@@ -778,7 +779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -837,7 +838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -851,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -866,7 +867,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="2">
         <v>0</v>
@@ -896,7 +897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -955,7 +956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1014,7 +1015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -1034,7 +1035,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2">
         <v>0</v>
@@ -1073,7 +1074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1132,7 +1133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -1146,7 +1147,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -1191,7 +1192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1250,7 +1251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1309,7 +1310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -1365,10 +1366,10 @@
         <v>0</v>
       </c>
       <c r="S15" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
@@ -1427,7 +1428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1486,7 +1487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1545,7 +1546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -1589,7 +1590,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P19" s="2">
         <v>0</v>
@@ -1620,7 +1621,121 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0CFC16F-2116-4C71-B60E-F8CD089D0AD1}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="8.85546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B2:E5">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009262A543AE2C984FB0E2FE06670DE161" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e51fc58191cada46128d6653faa18bde">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="97c3d6fa-0fa7-4b8a-8b65-7af9a8bc3877" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a28107f629881f83bf5d11058b02ca3a" ns2:_="">
     <xsd:import namespace="97c3d6fa-0fa7-4b8a-8b65-7af9a8bc3877"/>
@@ -1798,16 +1913,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD127F84-9CD2-40B0-B72C-D5C37497C4DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{906E764F-7DB5-428A-ABDB-D87EEF8E5248}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1823,12 +1937,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD127F84-9CD2-40B0-B72C-D5C37497C4DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>